<commit_message>
all SOC crops run!
</commit_message>
<xml_diff>
--- a/data/crops/rothc_support/permcrops_baseline_rothc_scenarios_FAOGAEZ.xlsx
+++ b/data/crops/rothc_support/permcrops_baseline_rothc_scenarios_FAOGAEZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/rothc_support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="11_9BC43EBF71FB3192BEA8278AF65FF74D9D56121C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70E7F683-0C5A-4707-8A66-F1D3EF33C15B}"/>
+  <xr:revisionPtr revIDLastSave="212" documentId="11_9BC43EBF71FB3192BEA8278AF65FF74D9D56121C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9D8AAEC-AC02-48AF-987B-D4B903BAF0AE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1551" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="551">
   <si>
     <t>lu_fp</t>
   </si>
@@ -2427,7 +2427,7 @@
         <v>445</v>
       </c>
       <c r="T2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" s="11" t="s">
         <v>548</v>
@@ -2494,7 +2494,7 @@
         <v>414</v>
       </c>
       <c r="T3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U3" s="11" t="s">
         <v>548</v>
@@ -2561,7 +2561,7 @@
         <v>424</v>
       </c>
       <c r="T4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" s="11" t="s">
         <v>548</v>
@@ -2628,7 +2628,7 @@
         <v>430</v>
       </c>
       <c r="T5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U5" s="11" t="s">
         <v>548</v>
@@ -2695,7 +2695,7 @@
         <v>427</v>
       </c>
       <c r="T6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6" s="11" t="s">
         <v>548</v>
@@ -2762,7 +2762,7 @@
         <v>445</v>
       </c>
       <c r="T7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7" s="11" t="s">
         <v>548</v>
@@ -2829,7 +2829,7 @@
         <v>475</v>
       </c>
       <c r="T8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U8" s="11" t="s">
         <v>548</v>
@@ -2896,7 +2896,7 @@
         <v>479</v>
       </c>
       <c r="T9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U9" s="11" t="s">
         <v>548</v>
@@ -2963,7 +2963,7 @@
         <v>445</v>
       </c>
       <c r="T10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U10" s="11" t="s">
         <v>548</v>
@@ -3027,7 +3027,7 @@
         <v>445</v>
       </c>
       <c r="T11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U11" s="11" t="s">
         <v>548</v>
@@ -3068,9 +3068,7 @@
       <c r="I12" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="J12" s="8" t="s">
-        <v>380</v>
-      </c>
+      <c r="J12" s="8"/>
       <c r="M12" t="b">
         <v>0</v>
       </c>
@@ -3135,9 +3133,7 @@
       <c r="I13" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="J13" s="6" t="s">
-        <v>380</v>
-      </c>
+      <c r="J13" s="6"/>
       <c r="M13" t="b">
         <v>0</v>
       </c>
@@ -3202,9 +3198,7 @@
       <c r="I14" s="7" t="s">
         <v>387</v>
       </c>
-      <c r="J14" s="8" t="s">
-        <v>380</v>
-      </c>
+      <c r="J14" s="8"/>
       <c r="M14" t="b">
         <v>0</v>
       </c>
@@ -3269,9 +3263,7 @@
       <c r="I15" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="J15" s="6" t="s">
-        <v>380</v>
-      </c>
+      <c r="J15" s="6"/>
       <c r="M15" t="b">
         <v>0</v>
       </c>
@@ -3400,9 +3392,7 @@
       <c r="I17" s="7" t="s">
         <v>393</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>380</v>
-      </c>
+      <c r="J17" s="8"/>
       <c r="M17" t="b">
         <v>0</v>
       </c>
@@ -3467,9 +3457,7 @@
       <c r="I18" s="5" t="s">
         <v>396</v>
       </c>
-      <c r="J18" s="6" t="s">
-        <v>380</v>
-      </c>
+      <c r="J18" s="6"/>
       <c r="M18" t="b">
         <v>0</v>
       </c>
@@ -3534,9 +3522,7 @@
       <c r="I19" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="J19" s="8" t="s">
-        <v>380</v>
-      </c>
+      <c r="J19" s="8"/>
       <c r="M19" t="b">
         <v>0</v>
       </c>
@@ -3668,9 +3654,7 @@
       <c r="I21" s="7" t="s">
         <v>406</v>
       </c>
-      <c r="J21" s="8" t="s">
-        <v>380</v>
-      </c>
+      <c r="J21" s="8"/>
       <c r="M21" t="b">
         <v>0</v>
       </c>

</xml_diff>